<commit_message>
重构 Hu_YQ_2026_ChinaSciData 的 Exp1/Exp2 数据
- Exp1：Clean 对齐模板 v2（21 列），>50MB 拆分为 part1/part2；新增 raw 表；subj_info 改标准结构
- Exp2：Clean 重构（Session 阶段名、Phase、TrialType→Matching），合并为单文件（18 列）；新增 raw 表；subj_info 改标准结构
- 更新两实验的 JSON 与 Codebook；重写 clean.R
</commit_message>
<xml_diff>
--- a/1_Data/Hu_YQ_2026_ChinaSciData/Exp1/Codebook_Hu_YQ_2026_ChinaSciData_Exp1_Clean.xlsx
+++ b/1_Data/Hu_YQ_2026_ChinaSciData/Exp1/Codebook_Hu_YQ_2026_ChinaSciData_Exp1_Clean.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t xml:space="preserve">Variable_name</t>
   </si>
@@ -32,40 +32,31 @@
     <t xml:space="preserve">Participant ID</t>
   </si>
   <si>
-    <t xml:space="preserve">6001 - 6036</t>
+    <t xml:space="preserve">6001-6036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categorical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session number (training time point / lab visit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number (1-6; 7 = subject 6031 only)</t>
   </si>
   <si>
     <t xml:space="preserve">Numerical</t>
   </si>
   <si>
-    <t xml:space="preserve">Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Between-subjects group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">control; depression</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Categorical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Session</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Session number (one complete experimental participation)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 - 7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Task</t>
   </si>
   <si>
-    <t xml:space="preserve">Association/task type (whether the association involves a self-referential identity)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">emotion; reward; self-matching; NA</t>
+    <t xml:space="preserve">Task type: matching (self/emotion/reward associations) vs self-matching (self/friend/stranger association)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matching; self-matching</t>
   </si>
   <si>
     <t xml:space="preserve">Phase</t>
@@ -74,22 +65,31 @@
     <t xml:space="preserve">Trial phase</t>
   </si>
   <si>
-    <t xml:space="preserve">main; practice</t>
+    <t xml:space="preserve">practice; main</t>
   </si>
   <si>
     <t xml:space="preserve">Block</t>
   </si>
   <si>
-    <t xml:space="preserve">Block number (NA for practice trials)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 - 2</t>
+    <t xml:space="preserve">Block number (global 1-6 across sub-tasks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number (1-6); NA = practice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trial order within block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number (1-96 matching; 1-240 self-matching); NA = practice</t>
   </si>
   <si>
     <t xml:space="preserve">Matching</t>
   </si>
   <si>
-    <t xml:space="preserve">Whether the presented shape-label pair matches the learned association</t>
+    <t xml:space="preserve">Whether the presented shape-label pair matches the learned association (Matching) or not (Nonmatching)</t>
   </si>
   <si>
     <t xml:space="preserve">Matching; Nonmatching</t>
@@ -98,64 +98,79 @@
     <t xml:space="preserve">Shape</t>
   </si>
   <si>
-    <t xml:space="preserve">Presented shape stimulus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circle; Diamond; Pentagon; Square; Trapezoid; Triangle; NA</t>
+    <t xml:space="preserve">Shape stimulus image filename</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C.bmp; D.bmp; P.bmp; S.bmp; T.bmp; Tra.bmp; c.bmp; c_eh.bmp; c_en.bmp; c_es.bmp; hc.bmp; hc_eh.bmp; hc_en.bmp; hc_es.bmp; vc.bmp; vc_eh.bmp; vc_en.bmp; vc_es.bmp</t>
   </si>
   <si>
     <t xml:space="preserve">Shape_Origin_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">Identity of the shape in its original form</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1; 16; happy; neutral; other; self; NA</t>
+    <t xml:space="preserve">Original-language identity of the shape stimulus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">你; 生人; 高兴; 中性; ￥1; ￥16; 自己; 朋友</t>
   </si>
   <si>
     <t xml:space="preserve">Shape_English_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">English translation of the shape identity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Happy; High_reward; Low_reward; Neutral; Other; Self; NA</t>
+    <t xml:space="preserve">English identity of the shape stimulus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self; other; happy; neutral; 1; 16; friend; stranger</t>
   </si>
   <si>
     <t xml:space="preserve">Shape_Standardized_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">Canonical standardized identity of the shape (6-category vocabulary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Happy; High_reward; Low_reward; Neutral; Self; Stranger; NA</t>
+    <t xml:space="preserve">Standardized identity (6-category vocabulary: Self/Close/Stranger/NonPerson/Acquaintance/Celebrity; non-identity stimuli kept as-is)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self; Stranger; happy; neutral; ￥1; ￥16; Close</t>
   </si>
   <si>
     <t xml:space="preserve">Label</t>
   </si>
   <si>
-    <t xml:space="preserve">Presented label stimulus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">￥1; ￥16; 中性; 生人; 你; 高兴; NA</t>
+    <t xml:space="preserve">Label word presented (original language)</t>
   </si>
   <si>
     <t xml:space="preserve">Label_Origin_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">Identity of the label in its original form</t>
+    <t xml:space="preserve">Original-language identity of the label</t>
   </si>
   <si>
     <t xml:space="preserve">Label_English_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">English translation of the label identity</t>
+    <t xml:space="preserve">English identity of the label</t>
   </si>
   <si>
     <t xml:space="preserve">Label_Standardized_Identity</t>
   </si>
   <si>
-    <t xml:space="preserve">Canonical standardized identity of the label (6-category vocabulary)</t>
+    <t xml:space="preserve">Standardized identity (6-category vocabulary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extraIV1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valence: positive (self/happy/high-reward) vs neutral (other/neutral/low-reward)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">positive; neutral; NA (not applicable: self-matching task)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extraIV2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emotion embedded in the shape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">control; happy; neutral; sad; NA (not applicable: matching task)</t>
   </si>
   <si>
     <t xml:space="preserve">CorrResponse</t>
@@ -164,40 +179,34 @@
     <t xml:space="preserve">Correct response key</t>
   </si>
   <si>
-    <t xml:space="preserve">1; 2; NA</t>
+    <t xml:space="preserve">1; 2 (matching); m; n (self-matching)</t>
   </si>
   <si>
     <t xml:space="preserve">Response</t>
   </si>
   <si>
-    <t xml:space="preserve">Participant's response key (NA = no response)</t>
+    <t xml:space="preserve">Actual key response; NA = no response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1; 2 (matching); m; n (self-matching); NA (no response)</t>
   </si>
   <si>
     <t xml:space="preserve">RT_ms</t>
   </si>
   <si>
-    <t xml:space="preserve">Reaction time in milliseconds (NA = no response)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">milliseconds (NA = no response)</t>
+    <t xml:space="preserve">Reaction time in milliseconds; NA = no response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ms; NA = no response</t>
   </si>
   <si>
     <t xml:space="preserve">ACC</t>
   </si>
   <si>
-    <t xml:space="preserve">Accuracy: 1 = correct, 0 = incorrect (wrong key), NA = no response</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 (correct); 0 (incorrect); NA (no response)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clock.StartTimeOfDay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trial start time of day (MM/DD/YY HH:MM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10/21/15 19:21; 10/23/15 08:46; 10/23/15 15:54; 10/23/15 18:58; 10/24/15 09:11; 10/24/15 11:03; 10/24/15 13:52; 10/24/15 17:07; 10/24/15 18:44; 10/24/15 19:15; 10/25/15 07:59; 10/25/15 08:30; 10/25/15 10:11; 10/25/15 10:22; 10/25/15 15:05; 10/25/15 15:18; 10/25/15 18:51; 10/25/15 19:01; 10/26/15 08:26; 10/26/15 10:29; 10/26/15 13:49; 10/26/15 14:07; 10/26/15 20:05; 10/27/15 10:20; 10/29/15 07:59; 10/29/15 09:52; 10/29/15 10:11; 10/29/15 13:53; 10/29/15 13:55; 10/29/15 14:08; 10/29/15 18:49; 10/29/15 18:56; 10/29/15 19:02; 10/31/15 08:04; 10/31/15 08:22; 10/31/15 10:09; 10/31/15 14:01; 10/31/15 14:03; 10/31/15 16:00; 10/31/15 16:11</t>
+    <t xml:space="preserve">Accuracy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 (correct); 0 (error); NA (no response)</t>
   </si>
 </sst>
 </file>
@@ -242,19 +251,6 @@
   </cellStyles>
   <dxfs count="0"/>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:D21" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:D21"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Variable_name"/>
-    <tableColumn id="2" name="Variable_description"/>
-    <tableColumn id="3" name="Variable_value"/>
-    <tableColumn id="4" name="Variable_category"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -606,7 +602,7 @@
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -634,7 +630,7 @@
         <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -648,7 +644,7 @@
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +658,7 @@
         <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -676,7 +672,7 @@
         <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -690,7 +686,7 @@
         <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +700,7 @@
         <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -715,80 +711,80 @@
         <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="B14" t="s">
-        <v>43</v>
-      </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" t="s">
         <v>44</v>
-      </c>
-      <c r="B15" t="s">
-        <v>45</v>
       </c>
       <c r="C15" t="s">
         <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
         <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>47</v>
       </c>
       <c r="C16" t="s">
         <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" t="s">
         <v>48</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>49</v>
       </c>
-      <c r="C17" t="s">
-        <v>50</v>
-      </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" t="s">
         <v>51</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>52</v>
       </c>
-      <c r="C18" t="s">
-        <v>50</v>
-      </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -816,7 +812,7 @@
         <v>58</v>
       </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -833,11 +829,22 @@
         <v>11</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>